<commit_message>
calc results for 0-shot without rows used in shots
</commit_message>
<xml_diff>
--- a/src/results/llm/one_shot_testing_01/results_for_presentation-one-shot.xlsx
+++ b/src/results/llm/one_shot_testing_01/results_for_presentation-one-shot.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\one_shot_testing_01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E80E3117-55F3-41E8-AF5F-ADF24F976F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6562B57-7424-4BBB-AAD7-99089205699F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="One-shot" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="15">
   <si>
     <t>Precision_positive</t>
   </si>
@@ -71,10 +71,16 @@
     <t>gemma4-26b-q4 v humanx one-shot with negative example</t>
   </si>
   <si>
-    <t>gemma4-26b-q4 v humanx ZERO-SHOT (original results)</t>
-  </si>
-  <si>
     <t>F1 macro diff</t>
+  </si>
+  <si>
+    <t>gemma4-26b-q4 v humanx ZERO-SHOT with 61 text (3 used in shots - removed)</t>
+  </si>
+  <si>
+    <t>gemma4-26b-q4 v humanx ZERO-SHOT with 62 texts (2 used in shots - removed)</t>
+  </si>
+  <si>
+    <t>gemma4-26b-q4 v humanx ZERO-SHOT with 64 texts (ORIGINAL RESULTS)</t>
   </si>
 </sst>
 </file>
@@ -162,30 +168,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -203,16 +207,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -492,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:W12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" style="2" customWidth="1"/>
@@ -501,14 +495,21 @@
     <col min="5" max="5" width="13.7109375" style="2" customWidth="1"/>
     <col min="6" max="6" width="14.5703125" style="2" customWidth="1"/>
     <col min="7" max="7" width="14.28515625" customWidth="1"/>
-    <col min="11" max="11" width="18" customWidth="1"/>
-    <col min="12" max="12" width="17" customWidth="1"/>
-    <col min="13" max="13" width="14.85546875" customWidth="1"/>
-    <col min="14" max="14" width="12.85546875" customWidth="1"/>
-    <col min="15" max="15" width="12.7109375" customWidth="1"/>
+    <col min="11" max="11" width="18" style="2" customWidth="1"/>
+    <col min="12" max="12" width="17" style="2" customWidth="1"/>
+    <col min="13" max="13" width="14.85546875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="12.85546875" style="2" customWidth="1"/>
+    <col min="15" max="15" width="12.7109375" style="2" customWidth="1"/>
+    <col min="17" max="17" width="3.28515625" customWidth="1"/>
+    <col min="18" max="18" width="14.28515625" customWidth="1"/>
+    <col min="19" max="19" width="20.140625" customWidth="1"/>
+    <col min="20" max="20" width="19.85546875" customWidth="1"/>
+    <col min="21" max="21" width="16.85546875" customWidth="1"/>
+    <col min="22" max="22" width="13" customWidth="1"/>
+    <col min="23" max="23" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>9</v>
       </c>
@@ -519,15 +520,23 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
       <c r="J1" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K1" s="5"/>
       <c r="L1" s="5"/>
       <c r="M1" s="5"/>
       <c r="N1" s="5"/>
       <c r="O1" s="5"/>
+      <c r="R1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="S1" s="5"/>
+      <c r="T1" s="5"/>
+      <c r="U1" s="5"/>
+      <c r="V1" s="5"/>
+      <c r="W1" s="5"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -546,8 +555,8 @@
       <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="7" t="s">
-        <v>12</v>
+      <c r="G2" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>5</v>
@@ -567,145 +576,225 @@
       <c r="O2" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="R2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="T2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="V2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W2" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="6">
+      <c r="B3" s="3">
         <v>0.85545335085413898</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="3">
         <v>0.95314787701317705</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="3">
         <v>0.90166204986149501</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="3">
         <v>0.869595326990244</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="3">
         <v>0.74044190704496304</v>
       </c>
-      <c r="G3" s="6">
+      <c r="G3" s="3">
         <f>E3-N3</f>
-        <v>1.7640073261080413E-3</v>
+        <v>6.940374947309591E-4</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="2">
+        <v>0.86369770580296901</v>
+      </c>
+      <c r="L3" s="2">
+        <v>0.93704245973645595</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0.898876404494382</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0.86890128949551304</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0.73849359928550096</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="S3" s="3">
         <v>0.86658195679796701</v>
       </c>
-      <c r="L3" s="9">
+      <c r="T3" s="3">
         <v>0.93681318681318604</v>
       </c>
-      <c r="M3" s="9">
+      <c r="U3" s="3">
         <v>0.90033003300329995</v>
       </c>
-      <c r="N3" s="9">
+      <c r="V3" s="3">
         <v>0.86783131966413596</v>
       </c>
-      <c r="O3" s="9">
+      <c r="W3" s="3">
         <v>0.73632332330032302</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="3">
         <v>0.65440210249671404</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="3">
         <v>0.93785310734463201</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="3">
         <v>0.77089783281733704</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="3">
         <v>0.741199403738103</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="3">
         <v>0.50226189198051197</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="3">
         <f t="shared" ref="G4:G5" si="0">E4-N4</f>
-        <v>-1.6229946230192027E-2</v>
+        <v>-1.1410118009914982E-2</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="2">
+        <v>0.66666666666666596</v>
+      </c>
+      <c r="L4" s="2">
+        <v>0.93032015065913298</v>
+      </c>
+      <c r="M4" s="2">
+        <v>0.77672955974842695</v>
+      </c>
+      <c r="N4" s="2">
+        <v>0.75260952174801798</v>
+      </c>
+      <c r="O4" s="2">
+        <v>0.52109249737380403</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="S4" s="3">
         <v>0.677255400254129</v>
       </c>
-      <c r="L4" s="9">
+      <c r="T4" s="3">
         <v>0.93508771929824497</v>
       </c>
-      <c r="M4" s="9">
+      <c r="U4" s="3">
         <v>0.78555637435519499</v>
       </c>
-      <c r="N4" s="9">
+      <c r="V4" s="3">
         <v>0.75742934996829503</v>
       </c>
-      <c r="O4" s="9">
+      <c r="W4" s="3">
         <v>0.530029272231755</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="3">
         <v>0.88699080157687205</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="3">
         <v>0.9</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="3">
         <v>0.89344804765056196</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="3">
         <v>0.84697185529987795</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="3">
         <v>0.69397407785826604</v>
       </c>
-      <c r="G5" s="6">
+      <c r="G5" s="3">
         <f t="shared" si="0"/>
-        <v>1.0917344854773914E-2</v>
+        <v>1.5221173863415927E-2</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="2">
+        <v>0.88529014844804299</v>
+      </c>
+      <c r="L5" s="2">
+        <v>0.87466666666666604</v>
+      </c>
+      <c r="M5" s="2">
+        <v>0.87994634473507705</v>
+      </c>
+      <c r="N5" s="2">
+        <v>0.83175068143646202</v>
+      </c>
+      <c r="O5" s="2">
+        <v>0.66352346614896296</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="S5" s="3">
         <v>0.89199491740787795</v>
       </c>
-      <c r="L5" s="9">
+      <c r="T5" s="3">
         <v>0.87969924812029998</v>
       </c>
-      <c r="M5" s="9">
+      <c r="U5" s="3">
         <v>0.88580441640378504</v>
       </c>
-      <c r="N5" s="9">
+      <c r="V5" s="3">
         <v>0.83605451044510404</v>
       </c>
-      <c r="O5" s="9">
+      <c r="W5" s="3">
         <v>0.67213857126683996</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="J8" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -724,89 +813,217 @@
       <c r="F9" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>12</v>
+      <c r="G9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="O9" s="1" t="s">
+        <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="6">
+      <c r="B10" s="3">
         <v>0.85356695869837296</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="3">
         <v>0.951185495118549</v>
       </c>
-      <c r="D10" s="6">
+      <c r="D10" s="3">
         <v>0.89973614775725597</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="3">
         <v>0.859391883402437</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="3">
         <v>0.72026084157967196</v>
       </c>
-      <c r="G10" s="6">
-        <f>E10-N3</f>
-        <v>-8.4394362616989627E-3</v>
+      <c r="G10" s="3">
+        <f>N10-E10</f>
+        <v>4.5144835080820345E-3</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.86692506459948304</v>
+      </c>
+      <c r="L10" s="2">
+        <v>0.93584379358437897</v>
+      </c>
+      <c r="M10" s="2">
+        <v>0.90006706908115297</v>
+      </c>
+      <c r="N10" s="2">
+        <v>0.86390636691051903</v>
+      </c>
+      <c r="O10" s="2">
+        <v>0.72849669441685905</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="6">
+      <c r="B11" s="3">
         <v>0.66708385481852295</v>
       </c>
-      <c r="C11" s="6">
+      <c r="C11" s="3">
         <v>0.94503546099290703</v>
       </c>
-      <c r="D11" s="6">
+      <c r="D11" s="3">
         <v>0.78209831254585405</v>
       </c>
-      <c r="E11" s="6">
+      <c r="E11" s="3">
         <v>0.74150232847836495</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="3">
         <v>0.50327255793350301</v>
       </c>
-      <c r="G11" s="6">
-        <f t="shared" ref="G11:G12" si="1">E11-N4</f>
-        <v>-1.5927021489930082E-2</v>
+      <c r="G11" s="3">
+        <f t="shared" ref="G11:G12" si="1">N11-E11</f>
+        <v>1.2879926947878095E-2</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K11" s="2">
+        <v>0.68087855297157596</v>
+      </c>
+      <c r="L11" s="2">
+        <v>0.93439716312056698</v>
+      </c>
+      <c r="M11" s="2">
+        <v>0.78774289985052304</v>
+      </c>
+      <c r="N11" s="2">
+        <v>0.75438225542624304</v>
+      </c>
+      <c r="O11" s="2">
+        <v>0.52417037884089102</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="6">
+      <c r="B12" s="3">
         <v>0.88610763454317898</v>
       </c>
-      <c r="C12" s="6">
+      <c r="C12" s="3">
         <v>0.90653008962868098</v>
       </c>
-      <c r="D12" s="6">
+      <c r="D12" s="3">
         <v>0.89620253164556896</v>
       </c>
-      <c r="E12" s="6">
+      <c r="E12" s="3">
         <v>0.84243116273000096</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="3">
         <v>0.68494558073848399</v>
       </c>
-      <c r="G12" s="6">
+      <c r="G12" s="3">
         <f t="shared" si="1"/>
-        <v>6.376652284896922E-3</v>
+        <v>-7.939711128104987E-3</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K12" s="2">
+        <v>0.89147286821705396</v>
+      </c>
+      <c r="L12" s="2">
+        <v>0.88348271446862903</v>
+      </c>
+      <c r="M12" s="2">
+        <v>0.887459807073955</v>
+      </c>
+      <c r="N12" s="2">
+        <v>0.83449145160189597</v>
+      </c>
+      <c r="O12" s="2">
+        <v>0.66899592486857695</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="R1:W1"/>
+    <mergeCell ref="A8:G8"/>
     <mergeCell ref="J1:O1"/>
-    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="J8:O8"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:A5 A2:G2">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A9:F9 A10:A12">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:F7 B9:F1048576 G2">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G1:G1048576">
+    <cfRule type="cellIs" dxfId="1" priority="11" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="12" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
     <cfRule type="colorScale" priority="14">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -818,31 +1035,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:F7 B9:F1048576 G2">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A9:F9 A10:A12">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="J2:J5">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J9:J12">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K2:O2">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -854,7 +1071,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:O2">
+  <conditionalFormatting sqref="K3:O3">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -866,7 +1083,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K3:O3">
+  <conditionalFormatting sqref="K4:O4">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -878,7 +1095,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K4:O4">
+  <conditionalFormatting sqref="K5:O5">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -890,19 +1107,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:O5">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
+  <conditionalFormatting sqref="K9:O9">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -914,7 +1119,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
+  <conditionalFormatting sqref="K10:O10">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -926,12 +1131,88 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G1:G1048576">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
-      <formula>0</formula>
+  <conditionalFormatting sqref="K11:O11">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K12:O12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R5">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:W2">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S3:W3">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S4:W4">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S5:W5">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Recalc metrics for one-shot
</commit_message>
<xml_diff>
--- a/src/results/llm/one_shot_testing_01/results_for_presentation-one-shot.xlsx
+++ b/src/results/llm/one_shot_testing_01/results_for_presentation-one-shot.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\one_shot_testing_01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6562B57-7424-4BBB-AAD7-99089205699F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A34740D5-1F0C-4145-AC99-7E99918F0DBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="One-shot" sheetId="1" r:id="rId1"/>
@@ -599,24 +599,24 @@
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3">
-        <v>0.85545335085413898</v>
-      </c>
-      <c r="C3" s="3">
-        <v>0.95314787701317705</v>
-      </c>
-      <c r="D3" s="3">
-        <v>0.90166204986149501</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0.869595326990244</v>
-      </c>
-      <c r="F3" s="3">
-        <v>0.74044190704496304</v>
+      <c r="B3" s="2">
+        <v>0.86096256684491901</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.94289897510980902</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.90006988120195597</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0.86942614691439402</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.73971866995623103</v>
       </c>
       <c r="G3" s="3">
         <f>E3-N3</f>
-        <v>6.940374947309591E-4</v>
+        <v>5.2485741888097515E-4</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>6</v>
@@ -659,24 +659,24 @@
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3">
-        <v>0.65440210249671404</v>
-      </c>
-      <c r="C4" s="3">
-        <v>0.93785310734463201</v>
-      </c>
-      <c r="D4" s="3">
-        <v>0.77089783281733704</v>
-      </c>
-      <c r="E4" s="3">
-        <v>0.741199403738103</v>
-      </c>
-      <c r="F4" s="3">
-        <v>0.50226189198051197</v>
+      <c r="B4" s="2">
+        <v>0.65775401069518702</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.92655367231638397</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.76935105551211802</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.74271210138454802</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.50303422312986401</v>
       </c>
       <c r="G4" s="3">
         <f t="shared" ref="G4:G5" si="0">E4-N4</f>
-        <v>-1.1410118009914982E-2</v>
+        <v>-9.8974203634699665E-3</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>7</v>
@@ -719,24 +719,24 @@
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3">
-        <v>0.88699080157687205</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0.9</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0.89344804765056196</v>
-      </c>
-      <c r="E5" s="3">
-        <v>0.84697185529987795</v>
-      </c>
-      <c r="F5" s="3">
-        <v>0.69397407785826604</v>
+      <c r="B5" s="2">
+        <v>0.88903743300000004</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.88666666699999996</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.88785046700000003</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.84148620925461504</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.68297345099999995</v>
       </c>
       <c r="G5" s="3">
         <f t="shared" si="0"/>
-        <v>1.5221173863415927E-2</v>
+        <v>9.7355278181530114E-3</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>8</v>
@@ -839,24 +839,24 @@
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="3">
-        <v>0.85356695869837296</v>
-      </c>
-      <c r="C10" s="3">
-        <v>0.951185495118549</v>
-      </c>
-      <c r="D10" s="3">
-        <v>0.89973614775725597</v>
-      </c>
-      <c r="E10" s="3">
-        <v>0.859391883402437</v>
-      </c>
-      <c r="F10" s="3">
-        <v>0.72026084157967196</v>
+      <c r="B10" s="2">
+        <v>0.85839598997493705</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.95536959553695899</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.90429042904290402</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.86593831796972798</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.73325025221055096</v>
       </c>
       <c r="G10" s="3">
-        <f>N10-E10</f>
-        <v>4.5144835080820345E-3</v>
+        <f>E10-N10</f>
+        <v>2.0319510592089474E-3</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>6</v>
@@ -881,24 +881,24 @@
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="3">
-        <v>0.66708385481852295</v>
-      </c>
-      <c r="C11" s="3">
-        <v>0.94503546099290703</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0.78209831254585405</v>
-      </c>
-      <c r="E11" s="3">
-        <v>0.74150232847836495</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0.50327255793350301</v>
+      <c r="B11" s="2">
+        <v>0.67293233082706705</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.95212765957446799</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0.78854625550660795</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.74940391246155302</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.518290708967303</v>
       </c>
       <c r="G11" s="3">
-        <f t="shared" ref="G11:G12" si="1">N11-E11</f>
-        <v>1.2879926947878095E-2</v>
+        <f t="shared" ref="G11:G12" si="1">E11-N11</f>
+        <v>-4.978342964690019E-3</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>7</v>
@@ -923,24 +923,24 @@
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="3">
-        <v>0.88610763454317898</v>
-      </c>
-      <c r="C12" s="3">
-        <v>0.90653008962868098</v>
-      </c>
-      <c r="D12" s="3">
-        <v>0.89620253164556896</v>
-      </c>
-      <c r="E12" s="3">
-        <v>0.84243116273000096</v>
-      </c>
-      <c r="F12" s="3">
-        <v>0.68494558073848399</v>
+      <c r="B12" s="2">
+        <v>0.88972431077694203</v>
+      </c>
+      <c r="C12" s="2">
+        <v>0.90909090909090895</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0.899303356554781</v>
+      </c>
+      <c r="E12" s="2">
+        <v>0.84733507596078805</v>
+      </c>
+      <c r="F12" s="2">
+        <v>0.69474205734811401</v>
       </c>
       <c r="G12" s="3">
         <f t="shared" si="1"/>
-        <v>-7.939711128104987E-3</v>
+        <v>1.2843624358892081E-2</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
One-shot metrics with json-repair
</commit_message>
<xml_diff>
--- a/src/results/llm/one_shot_testing_01/results_for_presentation-one-shot.xlsx
+++ b/src/results/llm/one_shot_testing_01/results_for_presentation-one-shot.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\one_shot_testing_01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{160EED19-90F9-4F33-B3F8-04DB116A7F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD285F5-370B-4909-B017-8949995963E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="15">
   <si>
     <t>Precision_positive</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>gemma4-26b-q4 v humanx ZERO-SHOT with 62 texts (2 used in shots - removed)</t>
-  </si>
-  <si>
-    <t>gemma4-26b-q4 v humanx ZERO-SHOT with 64 texts (ORIGINAL RESULTS)</t>
   </si>
   <si>
     <t>RESULTS AFTER PARSING RESPONSES WITH JSON-REPAIR</t>
@@ -192,15 +189,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -209,9 +209,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -221,21 +226,21 @@
   <dxfs count="2">
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -515,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W27"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.140625" style="2" customWidth="1"/>
@@ -538,8 +543,8 @@
     <col min="23" max="23" width="14.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="5"/>
@@ -556,16 +561,8 @@
       <c r="M1" s="5"/>
       <c r="N1" s="5"/>
       <c r="O1" s="5"/>
-      <c r="R1" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -605,26 +602,8 @@
       <c r="O2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="R2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="S2" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="T2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="V2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="W2" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -665,26 +644,8 @@
       <c r="O3" s="2">
         <v>0.73849359928550096</v>
       </c>
-      <c r="R3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="S3" s="3">
-        <v>0.86658195679796701</v>
-      </c>
-      <c r="T3" s="3">
-        <v>0.93681318681318604</v>
-      </c>
-      <c r="U3" s="3">
-        <v>0.90033003300329995</v>
-      </c>
-      <c r="V3" s="3">
-        <v>0.86783131966413596</v>
-      </c>
-      <c r="W3" s="3">
-        <v>0.73632332330032302</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
@@ -725,26 +686,8 @@
       <c r="O4" s="2">
         <v>0.52109249737380403</v>
       </c>
-      <c r="R4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="S4" s="3">
-        <v>0.677255400254129</v>
-      </c>
-      <c r="T4" s="3">
-        <v>0.93508771929824497</v>
-      </c>
-      <c r="U4" s="3">
-        <v>0.78555637435519499</v>
-      </c>
-      <c r="V4" s="3">
-        <v>0.75742934996829503</v>
-      </c>
-      <c r="W4" s="3">
-        <v>0.530029272231755</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -785,35 +728,17 @@
       <c r="O5" s="2">
         <v>0.66352346614896296</v>
       </c>
-      <c r="R5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="S5" s="3">
-        <v>0.89199491740787795</v>
-      </c>
-      <c r="T5" s="3">
-        <v>0.87969924812029998</v>
-      </c>
-      <c r="U5" s="3">
-        <v>0.88580441640378504</v>
-      </c>
-      <c r="V5" s="3">
-        <v>0.83605451044510404</v>
-      </c>
-      <c r="W5" s="3">
-        <v>0.67213857126683996</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
       <c r="J8" s="5" t="s">
         <v>13</v>
       </c>
@@ -823,7 +748,7 @@
       <c r="N8" s="5"/>
       <c r="O8" s="5"/>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
@@ -864,7 +789,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>6</v>
       </c>
@@ -906,7 +831,7 @@
         <v>0.72849669441685905</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
@@ -948,7 +873,7 @@
         <v>0.52417037884089102</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>8</v>
       </c>
@@ -990,60 +915,44 @@
         <v>0.66899592486857695</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="9"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="9"/>
-      <c r="T14" s="9"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
-      <c r="W14" s="9"/>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="9"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="9"/>
-      <c r="T15" s="9"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-      <c r="W15" s="9"/>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
+      <c r="I14" s="4"/>
+      <c r="J14" s="4"/>
+      <c r="K14" s="4"/>
+      <c r="L14" s="4"/>
+      <c r="M14" s="4"/>
+      <c r="N14" s="4"/>
+      <c r="O14" s="4"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
+      <c r="I15" s="4"/>
+      <c r="J15" s="4"/>
+      <c r="K15" s="4"/>
+      <c r="L15" s="4"/>
+      <c r="M15" s="4"/>
+      <c r="N15" s="4"/>
+      <c r="O15" s="4"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
       <c r="B16" s="5"/>
@@ -1060,16 +969,8 @@
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
-      <c r="R16" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="S16" s="5"/>
-      <c r="T16" s="5"/>
-      <c r="U16" s="5"/>
-      <c r="V16" s="5"/>
-      <c r="W16" s="5"/>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>5</v>
       </c>
@@ -1109,126 +1010,175 @@
       <c r="O17" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="R17" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="S17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="T17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="U17" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="V17" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="W17" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G18" s="3"/>
+      <c r="B18" s="2">
+        <v>0.86052631578947303</v>
+      </c>
+      <c r="C18" s="2">
+        <v>0.95754026354319099</v>
+      </c>
+      <c r="D18" s="2">
+        <v>0.90644490644490605</v>
+      </c>
+      <c r="E18" s="2">
+        <v>0.87607959607959596</v>
+      </c>
+      <c r="F18" s="2">
+        <v>0.75331755684030699</v>
+      </c>
+      <c r="G18" s="3">
+        <f>E18-N18</f>
+        <v>2.0340470340469707E-3</v>
+      </c>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
       <c r="J18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="R18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="S18" s="8">
-        <v>0.86759142496847397</v>
-      </c>
-      <c r="T18" s="8">
-        <v>0.94505494505494503</v>
-      </c>
-      <c r="U18" s="8">
-        <v>0.90466798159105799</v>
-      </c>
-      <c r="V18" s="8">
-        <v>0.87275111483504597</v>
-      </c>
-      <c r="W18" s="8">
-        <v>0.74627587318398403</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="K18" s="2">
+        <v>0.86479250334671998</v>
+      </c>
+      <c r="L18" s="2">
+        <v>0.94582723279648595</v>
+      </c>
+      <c r="M18" s="2">
+        <v>0.90349650349650301</v>
+      </c>
+      <c r="N18" s="2">
+        <v>0.87404554904554899</v>
+      </c>
+      <c r="O18" s="2">
+        <v>0.74890104369450206</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G19" s="3"/>
+      <c r="B19" s="2">
+        <v>0.65657894736842104</v>
+      </c>
+      <c r="C19" s="2">
+        <v>0.93973634651600702</v>
+      </c>
+      <c r="D19" s="2">
+        <v>0.77304415182029396</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0.74387358516039004</v>
+      </c>
+      <c r="F19" s="2">
+        <v>0.50723718673320195</v>
+      </c>
+      <c r="G19" s="3">
+        <f t="shared" ref="G19:G20" si="2">E19-N19</f>
+        <v>-1.3708875415027966E-2</v>
+      </c>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
       <c r="J19" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="R19" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="S19" s="8">
-        <v>0.679697351828499</v>
-      </c>
-      <c r="T19" s="8">
-        <v>0.94561403508771902</v>
-      </c>
-      <c r="U19" s="8">
-        <v>0.79090242112985998</v>
-      </c>
-      <c r="V19" s="8">
-        <v>0.76214905902143104</v>
-      </c>
-      <c r="W19" s="8">
-        <v>0.53999798244729103</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="K19" s="2">
+        <v>0.66934404283801796</v>
+      </c>
+      <c r="L19" s="2">
+        <v>0.94161958568738202</v>
+      </c>
+      <c r="M19" s="2">
+        <v>0.78247261345852803</v>
+      </c>
+      <c r="N19" s="2">
+        <v>0.757582460575418</v>
+      </c>
+      <c r="O19" s="2">
+        <v>0.53160688949363799</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G20" s="3"/>
+      <c r="B20" s="2">
+        <v>0.88815789473684204</v>
+      </c>
+      <c r="C20" s="2">
+        <v>0.9</v>
+      </c>
+      <c r="D20" s="2">
+        <v>0.89403973509933699</v>
+      </c>
+      <c r="E20" s="2">
+        <v>0.84800996655956995</v>
+      </c>
+      <c r="F20" s="2">
+        <v>0.69604484584241599</v>
+      </c>
+      <c r="G20" s="3">
+        <f t="shared" si="2"/>
+        <v>1.3037545062088984E-2</v>
+      </c>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
       <c r="J20" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="R20" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="S20" s="8">
-        <v>0.89155107187894</v>
-      </c>
-      <c r="T20" s="8">
-        <v>0.88596491228070096</v>
-      </c>
-      <c r="U20" s="8">
-        <v>0.88874921433060905</v>
-      </c>
-      <c r="V20" s="8">
-        <v>0.83914274034009595</v>
-      </c>
-      <c r="W20" s="8">
-        <v>0.67829149153697599</v>
-      </c>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="K20" s="2">
+        <v>0.88487282463186001</v>
+      </c>
+      <c r="L20" s="2">
+        <v>0.88133333333333297</v>
+      </c>
+      <c r="M20" s="2">
+        <v>0.88309953239812899</v>
+      </c>
+      <c r="N20" s="2">
+        <v>0.83497242149748097</v>
+      </c>
+      <c r="O20" s="2">
+        <v>0.66994725990727699</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+      <c r="G22" s="2"/>
+      <c r="H22" s="2"/>
+      <c r="I22" s="2"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="J23" s="5" t="s">
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="2"/>
+      <c r="I23" s="2"/>
+      <c r="J23" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="K23" s="11"/>
+      <c r="L23" s="11"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="11"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>5</v>
       </c>
@@ -1250,6 +1200,8 @@
       <c r="G24" s="1" t="s">
         <v>11</v>
       </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
       <c r="J24" s="1" t="s">
         <v>5</v>
       </c>
@@ -1269,46 +1221,149 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G25" s="3"/>
+      <c r="B25" s="2">
+        <v>0.85891089108910801</v>
+      </c>
+      <c r="C25" s="2">
+        <v>0.96792189679218898</v>
+      </c>
+      <c r="D25" s="2">
+        <v>0.910163934426229</v>
+      </c>
+      <c r="E25" s="2">
+        <v>0.87265116095559303</v>
+      </c>
+      <c r="F25" s="2">
+        <v>0.74695583729761705</v>
+      </c>
+      <c r="G25" s="3">
+        <f>E25-N25</f>
+        <v>3.6496733081989863E-3</v>
+      </c>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2"/>
       <c r="J25" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="K25" s="2">
+        <v>0.86794871794871797</v>
+      </c>
+      <c r="L25" s="2">
+        <v>0.94421199442119896</v>
+      </c>
+      <c r="M25" s="2">
+        <v>0.904475617902471</v>
+      </c>
+      <c r="N25" s="2">
+        <v>0.86900148764739404</v>
+      </c>
+      <c r="O25" s="2">
+        <v>0.73880914061022096</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G26" s="3"/>
+      <c r="B26" s="2">
+        <v>0.66831683168316802</v>
+      </c>
+      <c r="C26" s="2">
+        <v>0.95744680851063801</v>
+      </c>
+      <c r="D26" s="2">
+        <v>0.78717201166180695</v>
+      </c>
+      <c r="E26" s="2">
+        <v>0.74521202209106596</v>
+      </c>
+      <c r="F26" s="2">
+        <v>0.51194678713719699</v>
+      </c>
+      <c r="G26" s="3">
+        <f t="shared" ref="G26:G27" si="3">E26-N26</f>
+        <v>-1.4013580205188059E-2</v>
+      </c>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2"/>
       <c r="J26" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="K26" s="2">
+        <v>0.68333333333333302</v>
+      </c>
+      <c r="L26" s="2">
+        <v>0.94503546099290703</v>
+      </c>
+      <c r="M26" s="2">
+        <v>0.79315476190476097</v>
+      </c>
+      <c r="N26" s="2">
+        <v>0.75922560229625402</v>
+      </c>
+      <c r="O26" s="2">
+        <v>0.53442177334971097</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G27" s="3"/>
+      <c r="B27" s="2">
+        <v>0.88861386138613796</v>
+      </c>
+      <c r="C27" s="2">
+        <v>0.91933418693982005</v>
+      </c>
+      <c r="D27" s="2">
+        <v>0.90371302706104395</v>
+      </c>
+      <c r="E27" s="2">
+        <v>0.85211726972348201</v>
+      </c>
+      <c r="F27" s="2">
+        <v>0.70441134505187397</v>
+      </c>
+      <c r="G27" s="3">
+        <f t="shared" si="3"/>
+        <v>1.4437021213213996E-2</v>
+      </c>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2"/>
       <c r="J27" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="K27" s="2">
+        <v>0.89102564102564097</v>
+      </c>
+      <c r="L27" s="2">
+        <v>0.88988476312419895</v>
+      </c>
+      <c r="M27" s="2">
+        <v>0.89045483664317704</v>
+      </c>
+      <c r="N27" s="2">
+        <v>0.83768024851026801</v>
+      </c>
+      <c r="O27" s="2">
+        <v>0.67536075861646605</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A14:W15"/>
-    <mergeCell ref="R16:W16"/>
+  <mergeCells count="9">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="J1:O1"/>
+    <mergeCell ref="J8:O8"/>
     <mergeCell ref="A16:G16"/>
     <mergeCell ref="J16:O16"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="J23:O23"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="R1:W1"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="J1:O1"/>
-    <mergeCell ref="J8:O8"/>
+    <mergeCell ref="A14:O15"/>
   </mergeCells>
   <conditionalFormatting sqref="A2:A5 A2:G2">
     <cfRule type="colorScale" priority="46">
@@ -1322,6 +1377,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A17:A20 B17:G17">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A9:F9 A10:A12">
     <cfRule type="colorScale" priority="44">
       <colorScale>
@@ -1334,6 +1401,18 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A24:F24 A25:A27">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B2:F7 B9:F13 G2 B17:F22 B24:F1048576 G17">
     <cfRule type="colorScale" priority="45">
       <colorScale>
@@ -1346,26 +1425,48 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G9">
+    <cfRule type="colorScale" priority="36">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="35">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G1:G13 G16:G1048576">
-    <cfRule type="cellIs" dxfId="1" priority="33" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="34" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="34" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="0" priority="33" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9">
-    <cfRule type="colorScale" priority="35">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="36">
+  <conditionalFormatting sqref="G24">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>
@@ -1400,6 +1501,30 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J17:J20">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J24:J27">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="K2:O2">
     <cfRule type="colorScale" priority="31">
       <colorScale>
@@ -1486,196 +1611,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="K12:O12">
     <cfRule type="colorScale" priority="23">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R5">
-    <cfRule type="colorScale" priority="41">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:W2">
-    <cfRule type="colorScale" priority="40">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S3:W3">
-    <cfRule type="colorScale" priority="39">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S4:W4">
-    <cfRule type="colorScale" priority="38">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S5:W5">
-    <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R17:R20">
-    <cfRule type="colorScale" priority="22">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S17:W17">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S18:W18">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S19:W19">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S20:W20">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A17:A20 B17:G17">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A24:F24 A25:A27">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G24">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J17:J20">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J24:J27">
-    <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>